<commit_message>
add LCOM for methanol intersection case
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F449F1-FD44-4FBE-A0F9-53934BE4A4DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C60AE6E-EBD6-4051-900A-40D4B7009D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -724,19 +724,19 @@
         <v>13</v>
       </c>
       <c r="C2" s="2">
-        <v>69.595095364078418</v>
+        <v>79.071974149980875</v>
       </c>
       <c r="D2" s="2">
-        <v>384.70622159587788</v>
+        <v>437.09230155128313</v>
       </c>
       <c r="E2" s="2">
-        <v>1442189371.735008</v>
+        <v>1439202196.4283404</v>
       </c>
       <c r="F2" s="2">
-        <v>158965824.38942301</v>
+        <v>158923059.39427376</v>
       </c>
       <c r="G2" s="2">
-        <v>-133774104.9485403</v>
+        <v>-111623971.71011424</v>
       </c>
       <c r="H2" s="2">
         <v>2303240.7400001828</v>
@@ -759,20 +759,34 @@
       <c r="B3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="C3" s="2">
+        <v>78.310114411629584</v>
+      </c>
+      <c r="D3" s="2">
+        <v>432.88091021984127</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1724142064.7525234</v>
+      </c>
+      <c r="F3" s="2">
+        <v>146979029.99000928</v>
+      </c>
+      <c r="G3" s="2">
+        <v>-128127507.66122434</v>
+      </c>
+      <c r="H3" s="2">
+        <v>2303240.7400001828</v>
+      </c>
       <c r="I3" s="2">
         <f>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</f>
-        <v>0</v>
+        <v>416666.6665326964</v>
       </c>
       <c r="J3" s="2">
         <v>10.674776188588581</v>
       </c>
-      <c r="K3" s="2"/>
+      <c r="K3" s="2">
+        <v>560.58525239632695</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -904,10 +918,10 @@
         <v>46</v>
       </c>
       <c r="C2" s="2">
-        <v>69.595095364078418</v>
+        <v>79.071974149980875</v>
       </c>
       <c r="D2" s="2">
-        <v>384.70622159587788</v>
+        <v>437.09230155128313</v>
       </c>
       <c r="E2" s="2"/>
     </row>
@@ -918,12 +932,8 @@
       <c r="B3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="2">
-        <v>71.803044650000004</v>
-      </c>
-      <c r="D3" s="2">
-        <v>396.91127459357591</v>
-      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -933,12 +943,8 @@
       <c r="B4" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="2">
-        <v>70.625680473356155</v>
-      </c>
-      <c r="D4" s="2">
-        <v>390.40306709999999</v>
-      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -948,12 +954,8 @@
       <c r="B5" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="2">
-        <v>68.689400085859475</v>
-      </c>
-      <c r="D5" s="2">
-        <v>379.6997394</v>
-      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -963,12 +965,8 @@
       <c r="B6" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="2">
-        <v>67.890677236589767</v>
-      </c>
-      <c r="D6" s="2">
-        <v>375.28457689999999</v>
-      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -978,12 +976,8 @@
       <c r="B7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="2">
-        <v>65.639941548956116</v>
-      </c>
-      <c r="D7" s="2">
-        <v>362.84301022895181</v>
-      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -992,12 +986,8 @@
       <c r="B8" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="2">
-        <v>67.604029544370817</v>
-      </c>
-      <c r="D8" s="2">
-        <v>373.70005220000002</v>
-      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1006,12 +996,8 @@
       <c r="B9" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="2">
-        <v>71.612127255586572</v>
-      </c>
-      <c r="D9" s="2">
-        <v>395.85592566282571</v>
-      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -1020,12 +1006,8 @@
       <c r="B10" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="2">
-        <v>73.654120023996938</v>
-      </c>
-      <c r="D10" s="2">
-        <v>407.14360791042748</v>
-      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
@@ -1034,12 +1016,8 @@
       <c r="B11" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="2">
-        <v>62.613386021326697</v>
-      </c>
-      <c r="D11" s="2">
-        <v>346.11288384011141</v>
-      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1048,12 +1026,8 @@
       <c r="B12" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="2">
-        <v>66.035259580000002</v>
-      </c>
-      <c r="D12" s="2">
-        <v>365.02824045491485</v>
-      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -1062,12 +1036,8 @@
       <c r="B13" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="2">
-        <v>72.774571510000001</v>
-      </c>
-      <c r="D13" s="2">
-        <v>402.28165918679338</v>
-      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1076,12 +1046,8 @@
       <c r="B14" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="2">
-        <v>76.296108255634607</v>
-      </c>
-      <c r="D14" s="2">
-        <v>421.74793169999998</v>
-      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
@@ -1090,12 +1056,8 @@
       <c r="B15" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="2">
-        <v>68.136449838029762</v>
-      </c>
-      <c r="D15" s="2">
-        <v>376.64315327133113</v>
-      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1104,12 +1066,8 @@
       <c r="B16" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="2">
-        <v>69.361953979999996</v>
-      </c>
-      <c r="D16" s="2">
-        <v>383.41746782318944</v>
-      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
@@ -1118,12 +1076,8 @@
       <c r="B17" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="2">
-        <v>69.441196125889903</v>
-      </c>
-      <c r="D17" s="2">
-        <v>383.8555008070025</v>
-      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
@@ -1132,12 +1086,8 @@
       <c r="B18" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="2">
-        <v>69.246056331498551</v>
-      </c>
-      <c r="D18" s="2">
-        <v>382.77681139999999</v>
-      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
@@ -1146,12 +1096,8 @@
       <c r="B19" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="2">
-        <v>67.901620469999997</v>
-      </c>
-      <c r="D19" s="2">
-        <v>375.34506872240979</v>
-      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -1160,12 +1106,8 @@
       <c r="B20" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="2">
-        <v>68.748357918242007</v>
-      </c>
-      <c r="D20" s="2">
-        <v>380.02564515917106</v>
-      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
@@ -1174,12 +1116,8 @@
       <c r="B21" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="2">
-        <v>70.441836423490116</v>
-      </c>
-      <c r="D21" s="2">
-        <v>389.38681800762589</v>
-      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
@@ -1188,12 +1126,8 @@
       <c r="B22" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="2">
-        <v>71.288581789999995</v>
-      </c>
-      <c r="D22" s="2">
-        <v>394.06743824746638</v>
-      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
@@ -1202,12 +1136,8 @@
       <c r="B23" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="2">
-        <v>67.398683858444457</v>
-      </c>
-      <c r="D23" s="2">
-        <v>372.5649469</v>
-      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
@@ -1216,12 +1146,8 @@
       <c r="B24" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="2">
-        <v>68.312561592717216</v>
-      </c>
-      <c r="D24" s="2">
-        <v>377.6166599</v>
-      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
@@ -1230,12 +1156,8 @@
       <c r="B25" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="2">
-        <v>70.525455000029694</v>
-      </c>
-      <c r="D25" s="2">
-        <v>389.84904289999997</v>
-      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
@@ -1244,12 +1166,8 @@
       <c r="B26" t="s">
         <v>48</v>
       </c>
-      <c r="C26" s="2">
-        <v>155.42671709999999</v>
-      </c>
-      <c r="D26" s="2">
-        <v>859.16435278118581</v>
-      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
@@ -1258,12 +1176,8 @@
       <c r="B27" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="2">
-        <v>76.326256863212649</v>
-      </c>
-      <c r="D27" s="2">
-        <v>421.91458649999998</v>
-      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
@@ -1272,12 +1186,8 @@
       <c r="B28" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="2">
-        <v>72.740166950000003</v>
-      </c>
-      <c r="D28" s="2">
-        <v>402.09147844439104</v>
-      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
@@ -1286,12 +1196,8 @@
       <c r="B29" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C29" s="2">
-        <v>66.415629559999999</v>
-      </c>
-      <c r="D29" s="2">
-        <v>367.13084117418526</v>
-      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
@@ -1300,12 +1206,8 @@
       <c r="B30" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="6">
-        <v>63.062810195596832</v>
-      </c>
-      <c r="D30" s="6">
-        <v>348.5972008</v>
-      </c>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix bus in lifetime LCOM
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C60AE6E-EBD6-4051-900A-40D4B7009D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F596D461-7D0F-48A0-A939-1FD5A2C803B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -932,8 +932,12 @@
       <c r="B3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="C3" s="2">
+        <v>81.275350158925747</v>
+      </c>
+      <c r="D3" s="2">
+        <v>449.27207448961724</v>
+      </c>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -943,8 +947,12 @@
       <c r="B4" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="C4" s="2">
+        <v>80.100424630859479</v>
+      </c>
+      <c r="D4" s="2">
+        <v>442.77734726502871</v>
+      </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -954,8 +962,12 @@
       <c r="B5" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+      <c r="C5" s="2">
+        <v>78.168154818585222</v>
+      </c>
+      <c r="D5" s="2">
+        <v>432.09618913606829</v>
+      </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -965,8 +977,12 @@
       <c r="B6" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+      <c r="C6" s="2">
+        <v>77.371086346486052</v>
+      </c>
+      <c r="D6" s="2">
+        <v>427.6901717486312</v>
+      </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
fix bus in WACC LCOM
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F596D461-7D0F-48A0-A939-1FD5A2C803B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC92BC3B-4365-4942-BA6D-262C77439C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -992,8 +992,12 @@
       <c r="B7" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="C7" s="2">
+        <v>75.125012558461222</v>
+      </c>
+      <c r="D7" s="2">
+        <v>415.27437500000002</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
@@ -1002,8 +1006,12 @@
       <c r="B8" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="C8" s="2">
+        <v>77.085032381363334</v>
+      </c>
+      <c r="D8" s="2">
+        <v>426.10892899698064</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -1012,8 +1020,12 @@
       <c r="B9" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
+      <c r="C9" s="2">
+        <v>81.084828207442314</v>
+      </c>
+      <c r="D9" s="2">
+        <v>448.21891149999999</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
@@ -1022,8 +1034,12 @@
       <c r="B10" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+      <c r="C10" s="2">
+        <v>83.122591440887462</v>
+      </c>
+      <c r="D10" s="2">
+        <v>459.48321379823898</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">

</xml_diff>

<commit_message>
fix bus in investment cost LCOM
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC92BC3B-4365-4942-BA6D-262C77439C9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A35983F-518C-4E42-A8CC-DBBECCA7D322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -1048,8 +1048,12 @@
       <c r="B11" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
+      <c r="C11" s="2">
+        <v>72.161459216370218</v>
+      </c>
+      <c r="D11" s="2">
+        <v>398.89251066826864</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
@@ -1058,8 +1062,12 @@
       <c r="B12" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="C12" s="2">
+        <v>75.538100590500932</v>
+      </c>
+      <c r="D12" s="2">
+        <v>417.55783380000003</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
@@ -1068,8 +1076,12 @@
       <c r="B13" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="C13" s="2">
+        <v>81.990763985051061</v>
+      </c>
+      <c r="D13" s="2">
+        <v>453.22672313958782</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
@@ -1078,8 +1090,12 @@
       <c r="B14" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="C14" s="2">
+        <v>85.493573798602782</v>
+      </c>
+      <c r="D14" s="2">
+        <v>472.58947738672089</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">

</xml_diff>

<commit_message>
fix bug in efficiency and demand LCOM
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A35983F-518C-4E42-A8CC-DBBECCA7D322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E1BCC2-3A17-4533-8110-1744BA4AA963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -1104,8 +1104,12 @@
       <c r="B15" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="C15" s="2">
+        <v>78.171590251075841</v>
+      </c>
+      <c r="D15" s="2">
+        <v>432.115179443447</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1114,8 +1118,12 @@
       <c r="B16" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="C16" s="2">
+        <v>78.49222093533217</v>
+      </c>
+      <c r="D16" s="2">
+        <v>433.88755461475279</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
@@ -1124,8 +1132,12 @@
       <c r="B17" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="C17" s="2">
+        <v>79.716791605249099</v>
+      </c>
+      <c r="D17" s="2">
+        <v>440.65670915123803</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
@@ -1134,8 +1146,12 @@
       <c r="B18" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="C18" s="2">
+        <v>80.321920181700122</v>
+      </c>
+      <c r="D18" s="2">
+        <v>444.00172544884225</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
@@ -1224,8 +1240,12 @@
       <c r="B27" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
+      <c r="C27" s="2">
+        <v>88.81051338424885</v>
+      </c>
+      <c r="D27" s="2">
+        <v>490.92478231848668</v>
+      </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
@@ -1234,8 +1254,12 @@
       <c r="B28" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
+      <c r="C28" s="2">
+        <v>83.728374892272413</v>
+      </c>
+      <c r="D28" s="2">
+        <v>462.83185009895027</v>
+      </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
@@ -1244,8 +1268,12 @@
       <c r="B29" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
+      <c r="C29" s="2">
+        <v>74.988598312714814</v>
+      </c>
+      <c r="D29" s="2">
+        <v>414.52030733972907</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
@@ -1254,8 +1282,12 @@
       <c r="B30" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
+      <c r="C30" s="6">
+        <v>71.43077752774164</v>
+      </c>
+      <c r="D30" s="6">
+        <v>394.85346466723848</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix bug in co2 cost LCOM
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E1BCC2-3A17-4533-8110-1744BA4AA963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2DD555-F908-4B4D-9CFA-AC99BD40BE4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="50">
   <si>
     <t>run_name</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>variable cost</t>
+  </si>
+  <si>
+    <t>methanol escondida traif 10p down</t>
   </si>
 </sst>
 </file>
@@ -249,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -258,6 +261,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -338,8 +343,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}" name="Table3" displayName="Table3" ref="A1:D30" totalsRowShown="0">
-  <autoFilter ref="A1:D30" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}" name="Table3" displayName="Table3" ref="A1:D31" totalsRowShown="0">
+  <autoFilter ref="A1:D31" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8869914E-4BE8-401C-AC76-C6570071019E}" name="run_name"/>
     <tableColumn id="4" xr3:uid="{96123E5C-038E-4A38-8295-89FC853EE7AF}" name="type"/>
@@ -887,7 +892,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5837E54A-3435-47A0-958D-D2D4B44DC326}">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.453125" bestFit="1" customWidth="1"/>
@@ -1160,8 +1165,12 @@
       <c r="B19" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="C19" s="2">
+        <v>77.37849925829822</v>
+      </c>
+      <c r="D19" s="2">
+        <v>427.73114867781516</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -1170,8 +1179,12 @@
       <c r="B20" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="C20" s="2">
+        <v>78.225236704143668</v>
+      </c>
+      <c r="D20" s="2">
+        <v>432.41172511457188</v>
+      </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
@@ -1180,8 +1193,12 @@
       <c r="B21" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="C21" s="2">
+        <v>79.918713695686762</v>
+      </c>
+      <c r="D21" s="2">
+        <v>441.77288959560178</v>
+      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
@@ -1190,8 +1207,12 @@
       <c r="B22" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="C22" s="2">
+        <v>80.765459065707645</v>
+      </c>
+      <c r="D22" s="2">
+        <v>446.45350983543943</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
@@ -1288,6 +1309,14 @@
       <c r="D30" s="6">
         <v>394.85346466723848</v>
       </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B31" s="9"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix bug in power price LCOM
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2DD555-F908-4B4D-9CFA-AC99BD40BE4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB04A564-C69A-4AA5-A21C-B44A19D84134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -1221,8 +1221,12 @@
       <c r="B23" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="C23" s="2">
+        <v>75.68659190690758</v>
+      </c>
+      <c r="D23" s="2">
+        <v>418.37866081873909</v>
+      </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
@@ -1231,8 +1235,12 @@
       <c r="B24" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
+      <c r="C24" s="2">
+        <v>77.079263674147029</v>
+      </c>
+      <c r="D24" s="2">
+        <v>426.07704086542378</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
@@ -1241,8 +1249,12 @@
       <c r="B25" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+      <c r="C25" s="2">
+        <v>80.503301645795432</v>
+      </c>
+      <c r="D25" s="2">
+        <v>445.00436187536917</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
@@ -1251,8 +1263,12 @@
       <c r="B26" t="s">
         <v>48</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
+      <c r="C26" s="2">
+        <v>234.60011615233435</v>
+      </c>
+      <c r="D26" s="2">
+        <v>1296.8173087309592</v>
+      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">

</xml_diff>

<commit_message>
add preliminary sensitivities for grid tariffs
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB04A564-C69A-4AA5-A21C-B44A19D84134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B3BE46-FB5E-44CE-9702-40EB613DA1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
   <si>
     <t>run_name</t>
   </si>
@@ -186,7 +186,16 @@
     <t>variable cost</t>
   </si>
   <si>
-    <t>methanol escondida traif 10p down</t>
+    <t>methanol escondida traiff 10p down</t>
+  </si>
+  <si>
+    <t>methanol escondida traiff 05p down</t>
+  </si>
+  <si>
+    <t>methanol escondida traiff 05p up</t>
+  </si>
+  <si>
+    <t>methanol escondida traiff 10p up</t>
   </si>
 </sst>
 </file>
@@ -252,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -262,7 +271,6 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -343,8 +351,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}" name="Table3" displayName="Table3" ref="A1:D31" totalsRowShown="0">
-  <autoFilter ref="A1:D31" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}" name="Table3" displayName="Table3" ref="A1:D34" totalsRowShown="0">
+  <autoFilter ref="A1:D34" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8869914E-4BE8-401C-AC76-C6570071019E}" name="run_name"/>
     <tableColumn id="4" xr3:uid="{96123E5C-038E-4A38-8295-89FC853EE7AF}" name="type"/>
@@ -892,7 +900,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5837E54A-3435-47A0-958D-D2D4B44DC326}">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.453125" bestFit="1" customWidth="1"/>
@@ -1330,9 +1338,57 @@
       <c r="A31" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
+      <c r="B31" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="6">
+        <v>78.059428826878019</v>
+      </c>
+      <c r="D31" s="6">
+        <v>431.49517601524235</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" s="2">
+        <v>78.565701488429269</v>
+      </c>
+      <c r="D32" s="2">
+        <v>434.29373878326174</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" t="s">
+        <v>48</v>
+      </c>
+      <c r="C33" s="2">
+        <v>79.578246811532779</v>
+      </c>
+      <c r="D33" s="2">
+        <v>439.89086431930616</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" t="s">
+        <v>48</v>
+      </c>
+      <c r="C34" s="2">
+        <v>80.08451947308447</v>
+      </c>
+      <c r="D34" s="2">
+        <v>442.68942708732794</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
redo desalination and tariff sensitivity runs for methanol
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B3BE46-FB5E-44CE-9702-40EB613DA1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF56AB46-BCD1-45E7-8CD5-E4726F94ABF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Comparison_szenarios" sheetId="2" r:id="rId1"/>
+    <sheet name="Comparison_scenarios" sheetId="2" r:id="rId1"/>
     <sheet name="Comparison_sensitivities" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -261,16 +261,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -808,20 +806,34 @@
       <c r="B4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="C4" s="2">
+        <v>81.015948843836668</v>
+      </c>
+      <c r="D4" s="2">
+        <v>447.83816166454153</v>
+      </c>
+      <c r="E4" s="2">
+        <v>1789730808.6813896</v>
+      </c>
+      <c r="F4" s="2">
+        <v>149991159.26998231</v>
+      </c>
+      <c r="G4" s="2">
+        <v>-131051722.29205114</v>
+      </c>
+      <c r="H4" s="2">
+        <v>2303240.7400001828</v>
+      </c>
       <c r="I4" s="2">
         <f>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</f>
-        <v>0</v>
+        <v>416666.6665326964</v>
       </c>
       <c r="J4" s="2">
         <v>10.674776188588581</v>
       </c>
-      <c r="K4" s="2"/>
+      <c r="K4" s="2">
+        <v>560.58525239633184</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
@@ -1282,7 +1294,7 @@
       <c r="A27" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" t="s">
         <v>47</v>
       </c>
       <c r="C27" s="2">
@@ -1296,7 +1308,7 @@
       <c r="A28" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" t="s">
         <v>47</v>
       </c>
       <c r="C28" s="2">
@@ -1310,7 +1322,7 @@
       <c r="A29" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" t="s">
         <v>47</v>
       </c>
       <c r="C29" s="2">
@@ -1324,32 +1336,32 @@
       <c r="A30" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C30" s="6">
+      <c r="B30" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="2">
         <v>71.43077752774164</v>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="2">
         <v>394.85346466723848</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="6" t="s">
         <v>49</v>
       </c>
       <c r="B31" t="s">
         <v>48</v>
       </c>
-      <c r="C31" s="6">
+      <c r="C31" s="2">
         <v>78.059428826878019</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="2">
         <v>431.49517601524235</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="8" t="s">
+      <c r="A32" s="6" t="s">
         <v>50</v>
       </c>
       <c r="B32" t="s">
@@ -1363,7 +1375,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="6" t="s">
         <v>51</v>
       </c>
       <c r="B33" t="s">
@@ -1377,7 +1389,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="8" t="s">
+      <c r="A34" s="6" t="s">
         <v>52</v>
       </c>
       <c r="B34" t="s">

</xml_diff>

<commit_message>
add water supply sensitivities
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF56AB46-BCD1-45E7-8CD5-E4726F94ABF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{243CB332-AAA8-489F-ABE7-C16054BAB2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="57">
   <si>
     <t>run_name</t>
   </si>
@@ -186,16 +186,28 @@
     <t>variable cost</t>
   </si>
   <si>
-    <t>methanol escondida traiff 10p down</t>
-  </si>
-  <si>
-    <t>methanol escondida traiff 05p down</t>
-  </si>
-  <si>
-    <t>methanol escondida traiff 05p up</t>
-  </si>
-  <si>
-    <t>methanol escondida traiff 10p up</t>
+    <t>methanol escondida tariff 10p down</t>
+  </si>
+  <si>
+    <t>methanol escondida tariff 05p down</t>
+  </si>
+  <si>
+    <t>methanol escondida tariff 05p up</t>
+  </si>
+  <si>
+    <t>methanol escondida tariff 10p up</t>
+  </si>
+  <si>
+    <t>methanol escondida water 10p down</t>
+  </si>
+  <si>
+    <t>methanol escondida water 05p down</t>
+  </si>
+  <si>
+    <t>methanol escondida water 05p up</t>
+  </si>
+  <si>
+    <t>methanol escondida water 10p up</t>
   </si>
 </sst>
 </file>
@@ -302,13 +314,13 @@
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -331,31 +343,31 @@
   </sortState>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{6128FCF1-7EAF-4DB9-AB65-A4970FF7A7B8}" name="run_name"/>
-    <tableColumn id="9" xr3:uid="{E1E483D4-117D-4835-9726-D5751F56EFA1}" name="scenario" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{57DD338E-2930-40CB-AC06-11C7900CEBAE}" name="LCOE [Euro/MWh]" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{348EEC01-2159-40EC-A41A-F770A2113C35}" name="LCOE [Euro/t]" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{E1A32900-AFFC-4CA8-9A80-FDDFC927842B}" name="total_investment" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{9BDBD209-C39F-484C-957B-614102BD4B2E}" name="annual_costs" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{2F1A07E8-34B3-485A-A334-6B4F6D50721B}" name="annual_rev" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{B1C9F88F-C828-404D-9F5C-8363B244D4A6}" name="energy_production [MWh]" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{DFDA2CA3-CD6F-466B-81A4-84B9B62CB2C6}" name="energy_production [t]" dataDxfId="4">
+    <tableColumn id="9" xr3:uid="{E1E483D4-117D-4835-9726-D5751F56EFA1}" name="scenario" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{57DD338E-2930-40CB-AC06-11C7900CEBAE}" name="LCOE [Euro/MWh]" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{348EEC01-2159-40EC-A41A-F770A2113C35}" name="LCOE [Euro/t]" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{E1A32900-AFFC-4CA8-9A80-FDDFC927842B}" name="total_investment" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{9BDBD209-C39F-484C-957B-614102BD4B2E}" name="annual_costs" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{2F1A07E8-34B3-485A-A334-6B4F6D50721B}" name="annual_rev" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{B1C9F88F-C828-404D-9F5C-8363B244D4A6}" name="energy_production [MWh]" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{DFDA2CA3-CD6F-466B-81A4-84B9B62CB2C6}" name="energy_production [t]" dataDxfId="2">
       <calculatedColumnFormula>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{C340BB5F-846A-40DD-949F-DC14F9BEBD65}" name="pcf_value" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{3E078780-172C-4BE9-A08D-3FB4DFE536AE}" name="Size electrolyser" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{C340BB5F-846A-40DD-949F-DC14F9BEBD65}" name="pcf_value" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{3E078780-172C-4BE9-A08D-3FB4DFE536AE}" name="Size electrolyser" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}" name="Table3" displayName="Table3" ref="A1:D34" totalsRowShown="0">
-  <autoFilter ref="A1:D34" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}" name="Table3" displayName="Table3" ref="A1:D38" totalsRowShown="0">
+  <autoFilter ref="A1:D38" xr:uid="{1ED8C3B7-1CFE-4D76-BF2B-418405C32F6D}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8869914E-4BE8-401C-AC76-C6570071019E}" name="run_name"/>
     <tableColumn id="4" xr3:uid="{96123E5C-038E-4A38-8295-89FC853EE7AF}" name="type"/>
-    <tableColumn id="2" xr3:uid="{EDC23835-EE0F-4ABC-9DD3-CB899B7BD1E4}" name="LCOE [Euro/MWh]" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{7F3B94FF-49AD-4295-99F8-AE1E37B8E7F6}" name="LCOE [Euro/t]" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{EDC23835-EE0F-4ABC-9DD3-CB899B7BD1E4}" name="LCOE [Euro/MWh]" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{7F3B94FF-49AD-4295-99F8-AE1E37B8E7F6}" name="LCOE [Euro/t]" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -912,7 +924,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5837E54A-3435-47A0-958D-D2D4B44DC326}">
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.453125" bestFit="1" customWidth="1"/>
@@ -1402,6 +1414,62 @@
         <v>442.68942708732794</v>
       </c>
     </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="2">
+        <v>78.909203083368965</v>
+      </c>
+      <c r="D35" s="2">
+        <v>436.19253926640062</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" s="2">
+        <v>78.990588616660261</v>
+      </c>
+      <c r="D36" s="2">
+        <v>436.64242040876081</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B37" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37" s="2">
+        <v>79.153359683306576</v>
+      </c>
+      <c r="D37" s="2">
+        <v>437.54218269383352</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B38" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" s="2">
+        <v>79.23474521659314</v>
+      </c>
+      <c r="D38" s="2">
+        <v>437.99206383616757</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
add methanol local transport demand to LCOM comparison
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{243CB332-AAA8-489F-ABE7-C16054BAB2FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B79609F-6A21-499E-8B90-A13248770674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
   <sheets>
     <sheet name="Comparison_scenarios" sheetId="2" r:id="rId1"/>
     <sheet name="Comparison_sensitivities" sheetId="3" r:id="rId2"/>
+    <sheet name="comparison_with_transport" sheetId="4" r:id="rId3"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId4"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="69">
   <si>
     <t>run_name</t>
   </si>
@@ -208,13 +212,49 @@
   </si>
   <si>
     <t>methanol escondida water 10p up</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>energy demand from escondida to port</t>
+  </si>
+  <si>
+    <t>MWh/MWh methanol</t>
+  </si>
+  <si>
+    <t>energy demand from inters. to port</t>
+  </si>
+  <si>
+    <t>energy demand from inters. to escondida</t>
+  </si>
+  <si>
+    <t>energy demand from port to escondida</t>
+  </si>
+  <si>
+    <t>MWh/MWh ammonia</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>At Minera Escondida/Local Demand</t>
+  </si>
+  <si>
+    <t>At Puerto Coloso/Export</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -222,8 +262,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -236,8 +284,14 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -269,11 +323,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -281,11 +364,176 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="22">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
@@ -335,6 +583,76 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Input Parameters"/>
+      <sheetName val="Parameters"/>
+      <sheetName val="Demand Calculations"/>
+      <sheetName val="Transportation Calculations"/>
+      <sheetName val="CO2 Calculations"/>
+      <sheetName val="Scenarios &amp; Assumptions"/>
+      <sheetName val="Sources"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3">
+        <row r="10">
+          <cell r="B10">
+            <v>1.7085427135678392E-2</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="B11">
+            <v>1.0552763819095477E-2</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="B12">
+            <v>1.6331658291457288E-2</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="B13">
+            <v>4.2713567839195984E-2</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="B18">
+            <v>5.288888888888889E-3</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="B19">
+            <v>3.2666666666666664E-3</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="B20">
+            <v>2.0222222222222221E-3</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="B21">
+            <v>5.288888888888889E-3</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3A20CD82-EF7A-4E40-8E75-04BE9F55963D}" name="Table2" displayName="Table2" ref="A1:K7" totalsRowShown="0">
   <autoFilter ref="A1:K7" xr:uid="{3A20CD82-EF7A-4E40-8E75-04BE9F55963D}"/>
@@ -343,18 +661,18 @@
   </sortState>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{6128FCF1-7EAF-4DB9-AB65-A4970FF7A7B8}" name="run_name"/>
-    <tableColumn id="9" xr3:uid="{E1E483D4-117D-4835-9726-D5751F56EFA1}" name="scenario" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{57DD338E-2930-40CB-AC06-11C7900CEBAE}" name="LCOE [Euro/MWh]" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{348EEC01-2159-40EC-A41A-F770A2113C35}" name="LCOE [Euro/t]" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{E1A32900-AFFC-4CA8-9A80-FDDFC927842B}" name="total_investment" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{9BDBD209-C39F-484C-957B-614102BD4B2E}" name="annual_costs" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{2F1A07E8-34B3-485A-A334-6B4F6D50721B}" name="annual_rev" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{B1C9F88F-C828-404D-9F5C-8363B244D4A6}" name="energy_production [MWh]" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{DFDA2CA3-CD6F-466B-81A4-84B9B62CB2C6}" name="energy_production [t]" dataDxfId="2">
+    <tableColumn id="9" xr3:uid="{E1E483D4-117D-4835-9726-D5751F56EFA1}" name="scenario" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{57DD338E-2930-40CB-AC06-11C7900CEBAE}" name="LCOE [Euro/MWh]" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{348EEC01-2159-40EC-A41A-F770A2113C35}" name="LCOE [Euro/t]" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{E1A32900-AFFC-4CA8-9A80-FDDFC927842B}" name="total_investment" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{9BDBD209-C39F-484C-957B-614102BD4B2E}" name="annual_costs" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{2F1A07E8-34B3-485A-A334-6B4F6D50721B}" name="annual_rev" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{B1C9F88F-C828-404D-9F5C-8363B244D4A6}" name="energy_production [MWh]" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{DFDA2CA3-CD6F-466B-81A4-84B9B62CB2C6}" name="energy_production [t]" dataDxfId="12">
       <calculatedColumnFormula>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{C340BB5F-846A-40DD-949F-DC14F9BEBD65}" name="pcf_value" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{3E078780-172C-4BE9-A08D-3FB4DFE536AE}" name="Size electrolyser" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{C340BB5F-846A-40DD-949F-DC14F9BEBD65}" name="pcf_value" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{3E078780-172C-4BE9-A08D-3FB4DFE536AE}" name="Size electrolyser" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -366,8 +684,39 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8869914E-4BE8-401C-AC76-C6570071019E}" name="run_name"/>
     <tableColumn id="4" xr3:uid="{96123E5C-038E-4A38-8295-89FC853EE7AF}" name="type"/>
-    <tableColumn id="2" xr3:uid="{EDC23835-EE0F-4ABC-9DD3-CB899B7BD1E4}" name="LCOE [Euro/MWh]" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{7F3B94FF-49AD-4295-99F8-AE1E37B8E7F6}" name="LCOE [Euro/t]" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{EDC23835-EE0F-4ABC-9DD3-CB899B7BD1E4}" name="LCOE [Euro/MWh]" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{7F3B94FF-49AD-4295-99F8-AE1E37B8E7F6}" name="LCOE [Euro/t]" dataDxfId="20"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{82E022C4-2B02-4C7D-8C4E-E401A9CEA570}" name="Table1" displayName="Table1" ref="A1:E7" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+  <autoFilter ref="A1:E7" xr:uid="{82E022C4-2B02-4C7D-8C4E-E401A9CEA570}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{97253C94-9CD0-4EA9-9E0B-D2E8D1680665}" name="run_name" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{CDCCA758-A226-4144-A328-ACC22C8B55F3}" name="scenario"/>
+    <tableColumn id="3" xr3:uid="{AC1DE2CF-0DE6-4BB6-BF41-C459983F7708}" name="LCOE [Euro/MWh]" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{FE4D13C1-1034-49E7-9851-9BFFFDE27F2F}" name="At Minera Escondida/Local Demand" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{BCAB51B5-B2ED-4584-BE63-034E409FD08D}" name="At Puerto Coloso/Export" dataDxfId="0">
+      <calculatedColumnFormula>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C12</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{7F50A733-F3E7-4ECD-852B-68D82F47910A}" name="Table4" displayName="Table4" ref="A11:D19" totalsRowShown="0">
+  <autoFilter ref="A11:D19" xr:uid="{7F50A733-F3E7-4ECD-852B-68D82F47910A}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{AC055891-DBA2-45E9-AC8F-C4BA36A89FCD}" name="type"/>
+    <tableColumn id="2" xr3:uid="{1515481E-390E-40CF-BC98-1E1FECD3948F}" name="description" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{BC224235-A4F9-4FBE-B480-BF5C8A50D220}" name="value">
+      <calculatedColumnFormula>'[1]Transportation Calculations'!B14</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{E74EFA92-568A-4D1A-97C2-4879A00C50A1}" name="unit" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1476,4 +1825,266 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F630ECB-212C-4552-808B-85A59943E8A9}">
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+    <col min="4" max="4" width="33.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="9">
+        <v>79.071974149980875</v>
+      </c>
+      <c r="D2" s="9">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>79.071974149980875</v>
+      </c>
+      <c r="E2">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C12</f>
+        <v>80.422952602794624</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="11">
+        <v>78.310114411629584</v>
+      </c>
+      <c r="D3" s="11">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C14</f>
+        <v>79.589048440965243</v>
+      </c>
+      <c r="E3">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C13</f>
+        <v>79.136502553661856</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="9">
+        <v>81.015948843836668</v>
+      </c>
+      <c r="D4" s="9">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+C15*Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>84.476429070834712</v>
+      </c>
+      <c r="E4" s="2">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>81.015948843836668</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12">
+        <f>'[1]Transportation Calculations'!B10</f>
+        <v>1.7085427135678392E-2</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13">
+        <f>'[1]Transportation Calculations'!B11</f>
+        <v>1.0552763819095477E-2</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14">
+        <f>'[1]Transportation Calculations'!B12</f>
+        <v>1.6331658291457288E-2</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15">
+        <f>'[1]Transportation Calculations'!B13</f>
+        <v>4.2713567839195984E-2</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16">
+        <f>'[1]Transportation Calculations'!B18</f>
+        <v>5.288888888888889E-3</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17">
+        <f>'[1]Transportation Calculations'!B19</f>
+        <v>3.2666666666666664E-3</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18">
+        <f>'[1]Transportation Calculations'!B20</f>
+        <v>2.0222222222222221E-3</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19">
+        <f>'[1]Transportation Calculations'!B21</f>
+        <v>5.288888888888889E-3</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>63</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="E4" calculatedColumn="1"/>
+  </ignoredErrors>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
evaluation of the ammonia runs
</commit_message>
<xml_diff>
--- a/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
+++ b/Spine_Projects/03_output_data/03_runs_iaee_2026/03_evaluation/output_LCOE_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\03_output_data\03_runs_iaee_2026\03_evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B79609F-6A21-499E-8B90-A13248770674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A8C0159-874D-4FB3-AFE5-DC87C46227C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{3BB5C906-8FA9-43D8-B9CC-89F65EA8A47E}"/>
   </bookViews>
@@ -356,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -377,11 +377,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="22">
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -559,9 +565,6 @@
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -600,9 +603,9 @@
       <sheetName val="Sources"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
       <sheetData sheetId="3">
         <row r="10">
           <cell r="B10">
@@ -645,9 +648,9 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -668,11 +671,11 @@
     <tableColumn id="5" xr3:uid="{9BDBD209-C39F-484C-957B-614102BD4B2E}" name="annual_costs" dataDxfId="15"/>
     <tableColumn id="12" xr3:uid="{2F1A07E8-34B3-485A-A334-6B4F6D50721B}" name="annual_rev" dataDxfId="14"/>
     <tableColumn id="6" xr3:uid="{B1C9F88F-C828-404D-9F5C-8363B244D4A6}" name="energy_production [MWh]" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{DFDA2CA3-CD6F-466B-81A4-84B9B62CB2C6}" name="energy_production [t]" dataDxfId="12">
+    <tableColumn id="7" xr3:uid="{DFDA2CA3-CD6F-466B-81A4-84B9B62CB2C6}" name="energy_production [t]" dataDxfId="0">
       <calculatedColumnFormula>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{C340BB5F-846A-40DD-949F-DC14F9BEBD65}" name="pcf_value" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{3E078780-172C-4BE9-A08D-3FB4DFE536AE}" name="Size electrolyser" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{C340BB5F-846A-40DD-949F-DC14F9BEBD65}" name="pcf_value" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{3E078780-172C-4BE9-A08D-3FB4DFE536AE}" name="Size electrolyser" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -692,14 +695,14 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{82E022C4-2B02-4C7D-8C4E-E401A9CEA570}" name="Table1" displayName="Table1" ref="A1:E7" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{82E022C4-2B02-4C7D-8C4E-E401A9CEA570}" name="Table1" displayName="Table1" ref="A1:E7" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="9" tableBorderDxfId="10" totalsRowBorderDxfId="8">
   <autoFilter ref="A1:E7" xr:uid="{82E022C4-2B02-4C7D-8C4E-E401A9CEA570}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{97253C94-9CD0-4EA9-9E0B-D2E8D1680665}" name="run_name" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{97253C94-9CD0-4EA9-9E0B-D2E8D1680665}" name="run_name" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{CDCCA758-A226-4144-A328-ACC22C8B55F3}" name="scenario"/>
-    <tableColumn id="3" xr3:uid="{AC1DE2CF-0DE6-4BB6-BF41-C459983F7708}" name="LCOE [Euro/MWh]" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{FE4D13C1-1034-49E7-9851-9BFFFDE27F2F}" name="At Minera Escondida/Local Demand" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{BCAB51B5-B2ED-4584-BE63-034E409FD08D}" name="At Puerto Coloso/Export" dataDxfId="0">
+    <tableColumn id="3" xr3:uid="{AC1DE2CF-0DE6-4BB6-BF41-C459983F7708}" name="LCOE [Euro/MWh]" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{FE4D13C1-1034-49E7-9851-9BFFFDE27F2F}" name="At Minera Escondida/Local Demand" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{BCAB51B5-B2ED-4584-BE63-034E409FD08D}" name="At Puerto Coloso/Export" dataDxfId="1">
       <calculatedColumnFormula>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C12</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -712,11 +715,11 @@
   <autoFilter ref="A11:D19" xr:uid="{7F50A733-F3E7-4ECD-852B-68D82F47910A}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{AC055891-DBA2-45E9-AC8F-C4BA36A89FCD}" name="type"/>
-    <tableColumn id="2" xr3:uid="{1515481E-390E-40CF-BC98-1E1FECD3948F}" name="description" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{1515481E-390E-40CF-BC98-1E1FECD3948F}" name="description" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{BC224235-A4F9-4FBE-B480-BF5C8A50D220}" name="value">
       <calculatedColumnFormula>'[1]Transportation Calculations'!B14</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{E74EFA92-568A-4D1A-97C2-4879A00C50A1}" name="unit" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{E74EFA92-568A-4D1A-97C2-4879A00C50A1}" name="unit" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1168,16 +1171,16 @@
         <v>15</v>
       </c>
       <c r="C4" s="2">
-        <v>81.015948843836668</v>
+        <v>79.388116739869758</v>
       </c>
       <c r="D4" s="2">
-        <v>447.83816166454153</v>
+        <v>438.83986753428002</v>
       </c>
       <c r="E4" s="2">
         <v>1789730808.6813896</v>
       </c>
       <c r="F4" s="2">
-        <v>149991159.26998231</v>
+        <v>146241870.05024555</v>
       </c>
       <c r="G4" s="2">
         <v>-131051722.29205114</v>
@@ -1203,20 +1206,34 @@
       <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="C5" s="2">
+        <v>126.0234666741847</v>
+      </c>
+      <c r="D5" s="2">
+        <v>655.32202670576044</v>
+      </c>
+      <c r="E5" s="2">
+        <v>4647886836.9986534</v>
+      </c>
+      <c r="F5" s="2">
+        <v>162254145.38115364</v>
+      </c>
+      <c r="G5" s="2">
+        <v>-138201953.85988066</v>
+      </c>
+      <c r="H5" s="2">
+        <v>3645833.3333337754</v>
+      </c>
       <c r="I5" s="2">
-        <f>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</f>
-        <v>0</v>
+        <f>Table2[[#This Row],[energy_production '[MWh']]]/5.2</f>
+        <v>701121.79487187986</v>
       </c>
       <c r="J5" s="2">
         <v>10.674776188588581</v>
       </c>
-      <c r="K5" s="2"/>
+      <c r="K5" s="2">
+        <v>2815.8869332113072</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -1225,20 +1242,34 @@
       <c r="B6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="C6" s="2">
+        <v>128.76749001946612</v>
+      </c>
+      <c r="D6" s="2">
+        <v>669.59094810122383</v>
+      </c>
+      <c r="E6" s="2">
+        <v>5463144390.4983568</v>
+      </c>
+      <c r="F6" s="2">
+        <v>137559690.50524706</v>
+      </c>
+      <c r="G6" s="2">
+        <v>-179875579.42904782</v>
+      </c>
+      <c r="H6" s="2">
+        <v>3645833.3333337754</v>
+      </c>
       <c r="I6" s="2">
-        <f>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</f>
-        <v>0</v>
+        <f>Table2[[#This Row],[energy_production '[MWh']]]/5.2</f>
+        <v>701121.79487187986</v>
       </c>
       <c r="J6" s="2">
         <v>10.674776188588581</v>
       </c>
-      <c r="K6" s="2"/>
+      <c r="K6" s="2">
+        <v>483.22847566829876</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1247,20 +1278,34 @@
       <c r="B7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="C7" s="2">
+        <v>129.60081831905586</v>
+      </c>
+      <c r="D7" s="2">
+        <v>673.9242552590905</v>
+      </c>
+      <c r="E7" s="2">
+        <v>5474319313.9317894</v>
+      </c>
+      <c r="F7" s="2">
+        <v>137958458.4028241</v>
+      </c>
+      <c r="G7" s="2">
+        <v>-178283024.41761345</v>
+      </c>
+      <c r="H7" s="2">
+        <v>3645833.3333337754</v>
+      </c>
       <c r="I7" s="2">
-        <f>Table2[[#This Row],[energy_production '[MWh']]]*3.6/19.9</f>
-        <v>0</v>
+        <f>Table2[[#This Row],[energy_production '[MWh']]]/5.2</f>
+        <v>701121.79487187986</v>
       </c>
       <c r="J7" s="2">
         <v>10.6747761885886</v>
       </c>
-      <c r="K7" s="2"/>
+      <c r="K7" s="2">
+        <v>475.01275527802414</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1864,13 +1909,14 @@
         <v>13</v>
       </c>
       <c r="C2" s="9">
+        <f>Table2[[#This Row],[LCOE '[Euro/MWh']]]</f>
         <v>79.071974149980875</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="18">
         <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
         <v>79.071974149980875</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="19">
         <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C12</f>
         <v>80.422952602794624</v>
       </c>
@@ -1883,13 +1929,14 @@
         <v>14</v>
       </c>
       <c r="C3" s="11">
+        <f>Table2[[#This Row],[LCOE '[Euro/MWh']]]</f>
         <v>78.310114411629584</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="20">
         <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C14</f>
         <v>79.589048440965243</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="19">
         <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C13</f>
         <v>79.136502553661856</v>
       </c>
@@ -1902,15 +1949,16 @@
         <v>15</v>
       </c>
       <c r="C4" s="9">
-        <v>81.015948843836668</v>
-      </c>
-      <c r="D4" s="9">
+        <f>Table2[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>79.388116739869758</v>
+      </c>
+      <c r="D4" s="18">
         <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+C15*Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
-        <v>84.476429070834712</v>
-      </c>
-      <c r="E4" s="2">
+        <v>82.779066449864189</v>
+      </c>
+      <c r="E4" s="19">
         <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
-        <v>81.015948843836668</v>
+        <v>79.388116739869758</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -1920,8 +1968,18 @@
       <c r="B5" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
+      <c r="C5" s="11">
+        <f>Table2[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>126.0234666741847</v>
+      </c>
+      <c r="D5" s="11">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>126.0234666741847</v>
+      </c>
+      <c r="E5" s="11">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C16</f>
+        <v>126.68999078681706</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
@@ -1930,8 +1988,18 @@
       <c r="B6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
+      <c r="C6" s="9">
+        <f>Table2[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>128.76749001946612</v>
+      </c>
+      <c r="D6" s="11">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C18</f>
+        <v>129.02788649928326</v>
+      </c>
+      <c r="E6" s="11">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+Table1[[#This Row],[LCOE '[Euro/MWh']]]*C17</f>
+        <v>129.18813048686306</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="14" t="s">
@@ -1940,8 +2008,18 @@
       <c r="B7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
+      <c r="C7" s="16">
+        <f>Table2[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>129.60081831905586</v>
+      </c>
+      <c r="D7" s="11">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]+C19*Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>130.28626264705443</v>
+      </c>
+      <c r="E7" s="11">
+        <f>Table1[[#This Row],[LCOE '[Euro/MWh']]]</f>
+        <v>129.60081831905586</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">

</xml_diff>